<commit_message>
Reisekosten London: Flug als Position, Kilometer eingetragen, Eintrage-Box
Flug Frankfurt - London - Frankfurt als eigene Zeile in Block B ergaenzt,
Betrag offen. Kilometer nach Angabe eingetragen: 35 einfach, 70 hin und
zurueck, 21,00 EUR. Neue Uebersicht "Noch einzutragen" am Kopf der
Abrechnung, die je Feld die Zelle nennt und von fehlt auf erledigt springt,
sobald ein Betrag drinsteht.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-21-reisekosten-london-coldewey-holding.xlsx
+++ b/10_Output/2026-10-21-reisekosten-london-coldewey-holding.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Saetze 2026" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$I$77</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$I$83</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +29,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="C25" authorId="0">
+    <comment ref="C32" authorId="0">
       <text>
         <r>
           <rPr>
@@ -42,7 +42,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C26" authorId="0">
+    <comment ref="C33" authorId="0">
       <text>
         <r>
           <rPr>
@@ -54,7 +54,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C27" authorId="0">
+    <comment ref="C34" authorId="0">
       <text>
         <r>
           <rPr>
@@ -66,7 +66,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C28" authorId="0">
+    <comment ref="C35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -78,7 +78,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C44" authorId="0">
+    <comment ref="C51" authorId="0">
       <text>
         <r>
           <rPr>
@@ -91,7 +91,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D15" authorId="0">
+    <comment ref="D21" authorId="0">
       <text>
         <r>
           <rPr>
@@ -99,12 +99,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">OFFEN: gefahrene Kilometer hin und zurück eintragen.
-Die Entfernung konnte nicht verlässlich ermittelt werden, deshalb hier kein geschätzter Wert. Tacho oder Routenplaner, Wert dokumentieren.</t>
+          <t xml:space="preserve">35 km einfach laut Angabe Sascha, hin und zurück also 70 km.</t>
         </r>
       </text>
     </comment>
-    <comment ref="F33" authorId="0">
+    <comment ref="F40" authorId="0">
       <text>
         <r>
           <rPr>
@@ -115,6 +114,18 @@
           <t xml:space="preserve">Gestellte Mahlzeit mit „x“ markieren:
 F = Frühstück, M = Mittagessen, A = Abendessen.
 Dazu zählt auch das im Hotelpreis enthaltene Frühstück.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I29" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Hier den tatsächlich gezahlten Betrag eintragen.</t>
         </r>
       </text>
     </comment>
@@ -158,7 +169,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="127">
   <si>
     <t xml:space="preserve">Reisekostenabrechnung</t>
   </si>
@@ -223,6 +234,36 @@
     <t xml:space="preserve">21.10.2026</t>
   </si>
   <si>
+    <t xml:space="preserve">Noch einzutragen — danach rechnet sich alles von selbst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feld</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betrag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelle I29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frankfurt → London → Frankfurt, gezahlter Preis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelle I51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Übernachtung 07. auf 08.10., ohne Frühstücksanteil</t>
+  </si>
+  <si>
     <t xml:space="preserve">A · Fahrt mit eigenem Fahrzeug</t>
   </si>
   <si>
@@ -241,9 +282,6 @@
     <t xml:space="preserve">€/km</t>
   </si>
   <si>
-    <t xml:space="preserve">Betrag</t>
-  </si>
-  <si>
     <t xml:space="preserve">07.10.2026</t>
   </si>
   <si>
@@ -265,6 +303,9 @@
     <t xml:space="preserve">Beschreibung</t>
   </si>
   <si>
+    <t xml:space="preserve">Frankfurt → London → Frankfurt</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flughafen-Parken</t>
   </si>
   <si>
@@ -340,9 +381,6 @@
     <t xml:space="preserve">Beleg-Nr.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotel London</t>
-  </si>
-  <si>
     <t xml:space="preserve">Beleg fehlt</t>
   </si>
   <si>
@@ -400,19 +438,13 @@
     <t xml:space="preserve">Du hast 06. auf 07.10. genannt. Die Kartenumsätze sprechen für 07. auf 08.10.: Abflug Frankfurt „Pier J NonSchengen T3“ am 07.10., Rückflug „WH Smith Heathrow T2“ und Parkhaus-Ausfahrt am 08.10. Die Abrechnung steht auf 07.–08.10. — bitte prüfen.</t>
   </si>
   <si>
-    <t xml:space="preserve">Entfernung Im Zuckergarten 28 → FRA Terminal 3 und zurück fehlt. Block A, gelb markiert. Bei 0,30 €/km sind das je 10 km rund 3 €.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hotel</t>
   </si>
   <si>
-    <t xml:space="preserve">Keine Hotelzahlung im Kontoauszug gefunden. Rechnung nachreichen, Block D.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kein Flugticket im Kontoauszug gefunden. Falls privat bezahlt, in Block B ergänzen.</t>
+    <t xml:space="preserve">Betrag in Block D eintragen. Im Kontoauszug dieses Kontos ist die Zahlung nicht — Rechnung beilegen. Enthält sie Frühstück, den Anteil herausrechnen und in Block C das „F“ setzen, das kürzt die Pauschale um 13,20 €.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betrag in Block B eintragen. Hat die Firma direkt gezahlt, gehört er nicht hierher, sondern unten in „abzüglich direkt von der Firma bezahlt“.</t>
   </si>
   <si>
     <t xml:space="preserve">TfL 30,68 €</t>
@@ -599,6 +631,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -614,14 +654,6 @@
     <font>
       <b val="true"/>
       <sz val="12"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -659,8 +691,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFCE4E4"/>
+        <fgColor rgb="FFFCE4E4"/>
+        <bgColor rgb="FFE8E8E8"/>
       </patternFill>
     </fill>
     <fill>
@@ -671,13 +703,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1D9"/>
-        <bgColor rgb="FFE8E8E8"/>
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFCE4E4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4E4"/>
+        <fgColor rgb="FFD9E1D9"/>
         <bgColor rgb="FFE8E8E8"/>
       </patternFill>
     </fill>
@@ -731,7 +763,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -764,23 +796,35 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -800,11 +844,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="168" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -812,39 +860,35 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -856,7 +900,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1128,7 +1172,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1288,552 +1332,553 @@
       <c r="B14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="I14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="7" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="B15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="C15" s="10" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D15" s="9"/>
-      <c r="E15" s="10" t="str">
-        <f aca="false">IF($D15="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C15,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
-        <v/>
-      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
       <c r="I15" s="11" t="str">
-        <f aca="false">IF($D15="","",$D15*$E15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="10" t="str">
-        <f aca="false">IF($D16="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C16,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
-        <v/>
-      </c>
+        <f aca="false">IF(N(I29)=0,"fehlt","erledigt")</f>
+        <v>fehlt</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
       <c r="I16" s="11" t="str">
-        <f aca="false">IF($D16="","",$D16*$E16)</f>
+        <f aca="false">IF(N(I51)=0,"fehlt","erledigt")</f>
+        <v>fehlt</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="E21" s="14" t="n">
+        <f aca="false">IF($D21="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C21,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
+        <v>0.3</v>
+      </c>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="15" t="n">
+        <f aca="false">IF($D21="","",$D21*$E21)</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="14" t="str">
+        <f aca="false">IF($D22="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C22,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
         <v/>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="10" t="str">
-        <f aca="false">IF($D17="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C17,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="15" t="str">
+        <f aca="false">IF($D22="","",$D22*$E22)</f>
         <v/>
       </c>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="11" t="str">
-        <f aca="false">IF($D17="","",$D17*$E17)</f>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="14" t="str">
+        <f aca="false">IF($D23="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C23,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
         <v/>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="10" t="str">
-        <f aca="false">IF($D18="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C18,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="15" t="str">
+        <f aca="false">IF($D23="","",$D23*$E23)</f>
         <v/>
       </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="11" t="str">
-        <f aca="false">IF($D18="","",$D18*$E18)</f>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="14" t="str">
+        <f aca="false">IF($D24="","",IFERROR(INDEX('Saetze 2026'!$C$15:$C$17,MATCH($C24,'Saetze 2026'!$A$15:$A$17,0)),'Saetze 2026'!$C$15))</f>
         <v/>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="15" t="n">
-        <f aca="false">SUM(I15:I18)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-    </row>
-    <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="17" t="n">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="17" t="n">
-        <v>8.26</v>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="15" t="str">
+        <f aca="false">IF($D24="","",$D24*$E24)</f>
+        <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="18" t="s">
+      <c r="A25" s="16"/>
+      <c r="B25" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
-      <c r="I25" s="17" t="n">
+      <c r="I25" s="18" t="n">
+        <f aca="false">SUM(I21:I24)</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="20"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="21" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="21" t="n">
+        <v>8.26</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="21" t="n">
         <v>30.68</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="17" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="21" t="n">
         <v>3.73</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="17" t="n">
-        <v>3.72</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="17" t="n">
-        <v>2.36</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="17"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="15" t="n">
-        <f aca="false">SUM(I23:I29)</f>
-        <v>134.75</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
-    </row>
-    <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B33" s="7" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G33" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="H33" s="7" t="s">
+      <c r="C34" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="I33" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D34" s="11" t="n">
-        <f aca="false">IF($A34="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B34,'Saetze 2026'!$B$5:$B$7,0),MATCH($C34,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
-        <v>44</v>
-      </c>
-      <c r="E34" s="11" t="n">
-        <f aca="false">IF($A34="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B34,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F34)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G34)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H34)="x",'Saetze 2026'!$B$12,0)))</f>
-        <v>0</v>
-      </c>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
       <c r="F34" s="19"/>
       <c r="G34" s="19"/>
       <c r="H34" s="19"/>
-      <c r="I34" s="11" t="n">
-        <f aca="false">IF($A34="","",MAX(0,$D34-$E34))</f>
-        <v>44</v>
+      <c r="I34" s="21" t="n">
+        <v>3.72</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="s">
-        <v>37</v>
+      <c r="A35" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="B35" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D35" s="11" t="n">
-        <f aca="false">IF($A35="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B35,'Saetze 2026'!$B$5:$B$7,0),MATCH($C35,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
-        <v>44</v>
-      </c>
-      <c r="E35" s="11" t="n">
-        <f aca="false">IF($A35="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B35,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F35)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G35)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H35)="x",'Saetze 2026'!$B$12,0)))</f>
-        <v>0</v>
-      </c>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
       <c r="F35" s="19"/>
       <c r="G35" s="19"/>
       <c r="H35" s="19"/>
-      <c r="I35" s="11" t="n">
-        <f aca="false">IF($A35="","",MAX(0,$D35-$E35))</f>
-        <v>44</v>
+      <c r="I35" s="21" t="n">
+        <v>2.36</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8"/>
+      <c r="A36" s="12"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
-      <c r="D36" s="11" t="str">
-        <f aca="false">IF($A36="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B36,'Saetze 2026'!$B$5:$B$7,0),MATCH($C36,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
-        <v/>
-      </c>
-      <c r="E36" s="11" t="str">
-        <f aca="false">IF($A36="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B36,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F36)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G36)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H36)="x",'Saetze 2026'!$B$12,0)))</f>
-        <v/>
-      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
       <c r="F36" s="19"/>
       <c r="G36" s="19"/>
       <c r="H36" s="19"/>
-      <c r="I36" s="11" t="str">
-        <f aca="false">IF($A36="","",MAX(0,$D36-$E36))</f>
+      <c r="I36" s="21"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16"/>
+      <c r="B37" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="18" t="n">
+        <f aca="false">SUM(I29:I36)</f>
+        <v>134.75</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+    </row>
+    <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <f aca="false">IF($A41="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B41,'Saetze 2026'!$B$5:$B$7,0),MATCH($C41,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
+        <v>44</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <f aca="false">IF($A41="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B41,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F41)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G41)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H41)="x",'Saetze 2026'!$B$12,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="15" t="n">
+        <f aca="false">IF($A41="","",MAX(0,$D41-$E41))</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D42" s="15" t="n">
+        <f aca="false">IF($A42="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B42,'Saetze 2026'!$B$5:$B$7,0),MATCH($C42,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
+        <v>44</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <f aca="false">IF($A42="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B42,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F42)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G42)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H42)="x",'Saetze 2026'!$B$12,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="15" t="n">
+        <f aca="false">IF($A42="","",MAX(0,$D42-$E42))</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="15" t="str">
+        <f aca="false">IF($A43="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B43,'Saetze 2026'!$B$5:$B$7,0),MATCH($C43,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
         <v/>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="8"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="11" t="str">
-        <f aca="false">IF($A37="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B37,'Saetze 2026'!$B$5:$B$7,0),MATCH($C37,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
+      <c r="E43" s="15" t="str">
+        <f aca="false">IF($A43="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B43,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F43)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G43)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H43)="x",'Saetze 2026'!$B$12,0)))</f>
         <v/>
       </c>
-      <c r="E37" s="11" t="str">
-        <f aca="false">IF($A37="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B37,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F37)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G37)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H37)="x",'Saetze 2026'!$B$12,0)))</f>
+      <c r="F43" s="23"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="15" t="str">
+        <f aca="false">IF($A43="","",MAX(0,$D43-$E43))</f>
         <v/>
       </c>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="11" t="str">
-        <f aca="false">IF($A37="","",MAX(0,$D37-$E37))</f>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="12"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="15" t="str">
+        <f aca="false">IF($A44="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B44,'Saetze 2026'!$B$5:$B$7,0),MATCH($C44,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
         <v/>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="11" t="str">
-        <f aca="false">IF($A38="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B38,'Saetze 2026'!$B$5:$B$7,0),MATCH($C38,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
+      <c r="E44" s="15" t="str">
+        <f aca="false">IF($A44="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B44,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F44)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G44)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H44)="x",'Saetze 2026'!$B$12,0)))</f>
         <v/>
       </c>
-      <c r="E38" s="11" t="str">
-        <f aca="false">IF($A38="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B38,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F38)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G38)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H38)="x",'Saetze 2026'!$B$12,0)))</f>
+      <c r="F44" s="23"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="15" t="str">
+        <f aca="false">IF($A44="","",MAX(0,$D44-$E44))</f>
         <v/>
       </c>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="11" t="str">
-        <f aca="false">IF($A38="","",MAX(0,$D38-$E38))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="11" t="str">
-        <f aca="false">IF($A39="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B39,'Saetze 2026'!$B$5:$B$7,0),MATCH($C39,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
-        <v/>
-      </c>
-      <c r="E39" s="11" t="str">
-        <f aca="false">IF($A39="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B39,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F39)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G39)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H39)="x",'Saetze 2026'!$B$12,0)))</f>
-        <v/>
-      </c>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="11" t="str">
-        <f aca="false">IF($A39="","",MAX(0,$D39-$E39))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="15" t="n">
-        <f aca="false">SUM(I34:I39)</f>
-        <v>88</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-    </row>
-    <row r="43" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I43" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
-      <c r="F44" s="16"/>
-      <c r="G44" s="16"/>
-      <c r="H44" s="16"/>
-      <c r="I44" s="20"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="8"/>
+      <c r="A45" s="12"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="16"/>
-      <c r="G45" s="16"/>
-      <c r="H45" s="16"/>
-      <c r="I45" s="17"/>
+      <c r="D45" s="15" t="str">
+        <f aca="false">IF($A45="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B45,'Saetze 2026'!$B$5:$B$7,0),MATCH($C45,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
+        <v/>
+      </c>
+      <c r="E45" s="15" t="str">
+        <f aca="false">IF($A45="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B45,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F45)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G45)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H45)="x",'Saetze 2026'!$B$12,0)))</f>
+        <v/>
+      </c>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="15" t="str">
+        <f aca="false">IF($A45="","",MAX(0,$D45-$E45))</f>
+        <v/>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="8"/>
+      <c r="A46" s="12"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
-      <c r="F46" s="16"/>
-      <c r="G46" s="16"/>
-      <c r="H46" s="16"/>
-      <c r="I46" s="17"/>
+      <c r="D46" s="15" t="str">
+        <f aca="false">IF($A46="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B46,'Saetze 2026'!$B$5:$B$7,0),MATCH($C46,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
+        <v/>
+      </c>
+      <c r="E46" s="15" t="str">
+        <f aca="false">IF($A46="","",IFERROR(INDEX('Saetze 2026'!$C$5:$C$7,MATCH($B46,'Saetze 2026'!$B$5:$B$7,0)),0)*(IF(LOWER($F46)="x",'Saetze 2026'!$B$10,0)+IF(LOWER($G46)="x",'Saetze 2026'!$B$11,0)+IF(LOWER($H46)="x",'Saetze 2026'!$B$12,0)))</f>
+        <v/>
+      </c>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="15" t="str">
+        <f aca="false">IF($A46="","",MAX(0,$D46-$E46))</f>
+        <v/>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="13"/>
-      <c r="B47" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="15" t="n">
-        <f aca="false">SUM(I44:I46)</f>
-        <v>0</v>
+      <c r="A47" s="16"/>
+      <c r="B47" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="18" t="n">
+        <f aca="false">SUM(I41:I46)</f>
+        <v>88</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -1846,293 +1891,256 @@
     </row>
     <row r="50" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="I50" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="8" t="s">
-        <v>64</v>
+      <c r="A51" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D51" s="16"/>
-      <c r="E51" s="16"/>
-      <c r="F51" s="16"/>
-      <c r="G51" s="16"/>
-      <c r="H51" s="16"/>
-      <c r="I51" s="17" t="n">
-        <v>24.23</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19"/>
+      <c r="F51" s="19"/>
+      <c r="G51" s="19"/>
+      <c r="H51" s="19"/>
+      <c r="I51" s="20"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="8"/>
+      <c r="A52" s="12"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
-      <c r="D52" s="16"/>
-      <c r="E52" s="16"/>
-      <c r="F52" s="16"/>
-      <c r="G52" s="16"/>
-      <c r="H52" s="16"/>
-      <c r="I52" s="17"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="21"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="8"/>
+      <c r="A53" s="12"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
-      <c r="D53" s="16"/>
-      <c r="E53" s="16"/>
-      <c r="F53" s="16"/>
-      <c r="G53" s="16"/>
-      <c r="H53" s="16"/>
-      <c r="I53" s="17"/>
+      <c r="D53" s="19"/>
+      <c r="E53" s="19"/>
+      <c r="F53" s="19"/>
+      <c r="G53" s="19"/>
+      <c r="H53" s="19"/>
+      <c r="I53" s="21"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="8"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
+      <c r="A54" s="16"/>
+      <c r="B54" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C54" s="16"/>
       <c r="D54" s="16"/>
       <c r="E54" s="16"/>
       <c r="F54" s="16"/>
       <c r="G54" s="16"/>
       <c r="H54" s="16"/>
-      <c r="I54" s="17"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="13"/>
-      <c r="B55" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="13"/>
-      <c r="H55" s="13"/>
-      <c r="I55" s="15" t="n">
-        <f aca="false">SUM(I51:I54)</f>
+      <c r="I54" s="18" t="n">
+        <f aca="false">SUM(I51:I53)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="6"/>
+    </row>
+    <row r="57" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I57" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="19"/>
+      <c r="I58" s="21" t="n">
         <v>24.23</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
-      <c r="F57" s="6"/>
-      <c r="G57" s="6"/>
-      <c r="H57" s="6"/>
-      <c r="I57" s="6"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I58" s="21" t="n">
-        <f aca="false">I19+I30+I40+I47+I55</f>
-        <v>246.98</v>
-      </c>
-    </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="I59" s="17"/>
+      <c r="A59" s="12"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="19"/>
+      <c r="E59" s="19"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="19"/>
+      <c r="I59" s="21"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="I60" s="17"/>
-    </row>
-    <row r="61" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="23"/>
-      <c r="B61" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="C61" s="23"/>
-      <c r="D61" s="23"/>
-      <c r="E61" s="23"/>
-      <c r="F61" s="23"/>
-      <c r="G61" s="23"/>
-      <c r="H61" s="23"/>
-      <c r="I61" s="25" t="n">
-        <f aca="false">I58-N(I59)-N(I60)</f>
-        <v>246.98</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="E64" s="22" t="s">
-        <v>73</v>
-      </c>
+      <c r="A60" s="12"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="19"/>
+      <c r="E60" s="19"/>
+      <c r="F60" s="19"/>
+      <c r="G60" s="19"/>
+      <c r="H60" s="19"/>
+      <c r="I60" s="21"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="12"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="19"/>
+      <c r="E61" s="19"/>
+      <c r="F61" s="19"/>
+      <c r="G61" s="19"/>
+      <c r="H61" s="19"/>
+      <c r="I61" s="21"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="16"/>
+      <c r="B62" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C62" s="16"/>
+      <c r="D62" s="16"/>
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+      <c r="G62" s="16"/>
+      <c r="H62" s="16"/>
+      <c r="I62" s="18" t="n">
+        <f aca="false">SUM(I58:I61)</f>
+        <v>24.23</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B64" s="6"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="6"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B68" s="6"/>
-      <c r="C68" s="6"/>
-      <c r="D68" s="6"/>
-      <c r="E68" s="6"/>
-      <c r="F68" s="6"/>
-      <c r="G68" s="6"/>
-      <c r="H68" s="6"/>
-      <c r="I68" s="6"/>
-    </row>
-    <row r="69" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B69" s="27" t="s">
+      <c r="B65" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C69" s="28" t="s">
+      <c r="I65" s="24" t="n">
+        <f aca="false">I25+I37+I47+I54+I62</f>
+        <v>267.98</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="D69" s="28"/>
-      <c r="E69" s="28"/>
-      <c r="F69" s="28"/>
-      <c r="G69" s="28"/>
-      <c r="H69" s="28"/>
-      <c r="I69" s="28"/>
-    </row>
-    <row r="70" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B70" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="C70" s="28" t="s">
+      <c r="I66" s="21"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="D70" s="28"/>
-      <c r="E70" s="28"/>
-      <c r="F70" s="28"/>
-      <c r="G70" s="28"/>
-      <c r="H70" s="28"/>
-      <c r="I70" s="28"/>
-    </row>
-    <row r="71" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B71" s="27" t="s">
+      <c r="I67" s="21"/>
+    </row>
+    <row r="68" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="26"/>
+      <c r="B68" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="C71" s="28" t="s">
+      <c r="C68" s="26"/>
+      <c r="D68" s="26"/>
+      <c r="E68" s="26"/>
+      <c r="F68" s="26"/>
+      <c r="G68" s="26"/>
+      <c r="H68" s="26"/>
+      <c r="I68" s="28" t="n">
+        <f aca="false">I65-N(I66)-N(I67)</f>
+        <v>267.98</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="D71" s="28"/>
-      <c r="E71" s="28"/>
-      <c r="F71" s="28"/>
-      <c r="G71" s="28"/>
-      <c r="H71" s="28"/>
-      <c r="I71" s="28"/>
-    </row>
-    <row r="72" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B72" s="27" t="s">
+      <c r="E71" s="25" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C72" s="28" t="s">
+      <c r="E72" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D72" s="28"/>
-      <c r="E72" s="28"/>
-      <c r="F72" s="28"/>
-      <c r="G72" s="28"/>
-      <c r="H72" s="28"/>
-      <c r="I72" s="28"/>
-    </row>
-    <row r="73" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B73" s="27" t="s">
+    </row>
+    <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C73" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="D73" s="28"/>
-      <c r="E73" s="28"/>
-      <c r="F73" s="28"/>
-      <c r="G73" s="28"/>
-      <c r="H73" s="28"/>
-      <c r="I73" s="28"/>
-    </row>
-    <row r="74" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B74" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="C74" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="D74" s="28"/>
-      <c r="E74" s="28"/>
-      <c r="F74" s="28"/>
-      <c r="G74" s="28"/>
-      <c r="H74" s="28"/>
-      <c r="I74" s="28"/>
-    </row>
-    <row r="75" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="B75" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="C75" s="31" t="s">
-        <v>91</v>
-      </c>
-      <c r="D75" s="31"/>
-      <c r="E75" s="31"/>
-      <c r="F75" s="31"/>
-      <c r="G75" s="31"/>
-      <c r="H75" s="31"/>
-      <c r="I75" s="31"/>
+      <c r="B75" s="6"/>
+      <c r="C75" s="6"/>
+      <c r="D75" s="6"/>
+      <c r="E75" s="6"/>
+      <c r="F75" s="6"/>
+      <c r="G75" s="6"/>
+      <c r="H75" s="6"/>
+      <c r="I75" s="6"/>
     </row>
     <row r="76" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="29" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B76" s="30" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C76" s="31" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D76" s="31"/>
       <c r="E76" s="31"/>
@@ -2141,8 +2149,110 @@
       <c r="H76" s="31"/>
       <c r="I76" s="31"/>
     </row>
+    <row r="77" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B77" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="C77" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="D77" s="31"/>
+      <c r="E77" s="31"/>
+      <c r="F77" s="31"/>
+      <c r="G77" s="31"/>
+      <c r="H77" s="31"/>
+      <c r="I77" s="31"/>
+    </row>
+    <row r="78" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B78" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C78" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="D78" s="31"/>
+      <c r="E78" s="31"/>
+      <c r="F78" s="31"/>
+      <c r="G78" s="31"/>
+      <c r="H78" s="31"/>
+      <c r="I78" s="31"/>
+    </row>
+    <row r="79" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B79" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C79" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D79" s="31"/>
+      <c r="E79" s="31"/>
+      <c r="F79" s="31"/>
+      <c r="G79" s="31"/>
+      <c r="H79" s="31"/>
+      <c r="I79" s="31"/>
+    </row>
+    <row r="80" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B80" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C80" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="D80" s="31"/>
+      <c r="E80" s="31"/>
+      <c r="F80" s="31"/>
+      <c r="G80" s="31"/>
+      <c r="H80" s="31"/>
+      <c r="I80" s="31"/>
+    </row>
+    <row r="81" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B81" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="C81" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="D81" s="34"/>
+      <c r="E81" s="34"/>
+      <c r="F81" s="34"/>
+      <c r="G81" s="34"/>
+      <c r="H81" s="34"/>
+      <c r="I81" s="34"/>
+    </row>
+    <row r="82" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B82" s="33" t="s">
+        <v>99</v>
+      </c>
+      <c r="C82" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="D82" s="34"/>
+      <c r="E82" s="34"/>
+      <c r="F82" s="34"/>
+      <c r="G82" s="34"/>
+      <c r="H82" s="34"/>
+      <c r="I82" s="34"/>
+    </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="48">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="B4:E4"/>
@@ -2156,53 +2266,56 @@
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="A13:I13"/>
-    <mergeCell ref="E15:H15"/>
-    <mergeCell ref="E16:H16"/>
-    <mergeCell ref="E17:H17"/>
-    <mergeCell ref="E18:H18"/>
-    <mergeCell ref="A21:I21"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="C15:H15"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="E21:H21"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="E23:H23"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="A27:I27"/>
     <mergeCell ref="D29:H29"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A42:I42"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="A39:I39"/>
     <mergeCell ref="A49:I49"/>
     <mergeCell ref="D51:H51"/>
     <mergeCell ref="D52:H52"/>
     <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="A57:I57"/>
-    <mergeCell ref="A68:I68"/>
-    <mergeCell ref="C69:I69"/>
-    <mergeCell ref="C70:I70"/>
-    <mergeCell ref="C71:I71"/>
-    <mergeCell ref="C72:I72"/>
-    <mergeCell ref="C73:I73"/>
-    <mergeCell ref="C74:I74"/>
-    <mergeCell ref="C75:I75"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="A64:I64"/>
+    <mergeCell ref="A75:I75"/>
     <mergeCell ref="C76:I76"/>
+    <mergeCell ref="C77:I77"/>
+    <mergeCell ref="C78:I78"/>
+    <mergeCell ref="C79:I79"/>
+    <mergeCell ref="C80:I80"/>
+    <mergeCell ref="C81:I81"/>
+    <mergeCell ref="C82:I82"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C18" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C21:C24" type="list">
       <formula1>'Saetze 2026'!$A$15:$A$17</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B34:B39" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B41:B46" type="list">
       <formula1>'Saetze 2026'!$B$5:$B$7</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C34:C39" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C41:C46" type="list">
       <formula1>'Saetze 2026'!$C$4:$F$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F34:H39" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F41:H46" type="list">
       <formula1>"x"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2234,203 +2347,203 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="32" t="s">
-        <v>94</v>
+      <c r="A1" s="35" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="36" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="F5" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="36" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5" s="33" t="n">
-        <v>28</v>
-      </c>
-      <c r="D5" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="E5" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="F5" s="33" t="n">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>66</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>44</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>44</v>
+      </c>
+      <c r="F6" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="33" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="33" t="n">
-        <v>66</v>
-      </c>
-      <c r="D6" s="33" t="n">
-        <v>44</v>
-      </c>
-      <c r="E6" s="33" t="n">
-        <v>44</v>
-      </c>
-      <c r="F6" s="33" t="n">
+      <c r="G6" s="36" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="36" t="n">
+        <v>52</v>
+      </c>
+      <c r="D7" s="36" t="n">
+        <v>35</v>
+      </c>
+      <c r="E7" s="36" t="n">
+        <v>35</v>
+      </c>
+      <c r="F7" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="33" t="n">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>52</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>35</v>
-      </c>
-      <c r="E7" s="33" t="n">
-        <v>35</v>
-      </c>
-      <c r="F7" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="33" t="n">
+      <c r="G7" s="36" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>106</v>
-      </c>
-      <c r="B10" s="34" t="n">
+      <c r="A10" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" s="37" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="34" t="n">
+      <c r="A11" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="B11" s="37" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
-        <v>108</v>
-      </c>
-      <c r="B12" s="34" t="n">
+      <c r="A12" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="37" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="35" t="n">
+      <c r="A15" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="38" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="C16" s="35" t="n">
+      <c r="A16" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="C16" s="38" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" s="35" t="n">
+      <c r="A17" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="38" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reisekosten London: Datum korrigiert, Flugrechnung eingearbeitet
Reisedatum zurueck auf 06.-07.10.2026. Meine Korrektur auf 07.-08.10. anhand
der Kartenumsaetze war falsch: Haendler reichen Umsaetze ein bis zwei Tage
verzoegert ein, auch das Value Date ist nicht das Kaufdatum. Die Flugbuchung
LH 919 LHR-FRA am 07.10. um 19:30 belegt das urspruengliche Datum.

Flug Rueckreise 89,98 EUR aus Rechnung 2026-B2B7-000199110 eingetragen.
Rechnungsempfaenger ist die Coldewey Holding GmbH und im privaten Konto fehlt
die Zahlung, also direkt von der Firma gezahlt und unten wieder abgezogen.
Reisekosten gesamt 357,96 EUR, Erstattung an Sascha 267,98 EUR.

Fehlschluss und Regel daraus in wissen/reisekosten.md und wissen/feedback.md
festgehalten.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-21-reisekosten-london-coldewey-holding.xlsx
+++ b/10_Output/2026-10-21-reisekosten-london-coldewey-holding.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Saetze 2026" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$I$83</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$I$87</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +29,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="C32" authorId="0">
+    <comment ref="C33" authorId="0">
       <text>
         <r>
           <rPr>
@@ -39,18 +39,6 @@
           </rPr>
           <t xml:space="preserve">TfL bucht „Unpaid Fare“ nach, wenn beim Ein- oder Ausstieg nicht korrekt getappt wurde. Ist das eine reine Fahrpreis-Nachzahlung, ist sie absetzbar. Ist es ein Bußgeld (Penalty Fare), ist sie es nicht — dann Zeile löschen.
 Bitte den TfL-Kontoauszug prüfen.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C33" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">OFFEN: „About Town Business Services“ ließ sich nicht eindeutig zuordnen. Wenn das keine Reisekosten waren, Zeile löschen.</t>
         </r>
       </text>
     </comment>
@@ -78,6 +66,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="C36" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">OFFEN: „About Town Business Services“ ließ sich nicht eindeutig zuordnen. Wenn das keine Reisekosten waren, Zeile löschen.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="C51" authorId="0">
       <text>
         <r>
@@ -86,7 +86,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">OFFEN: Im hochgeladenen Kontoauszug ist für den 06.–08.10. keine Hotelzahlung zu finden. Entweder über ein anderes Konto oder vorab bezahlt.
+          <t xml:space="preserve">OFFEN: Im hochgeladenen Kontoauszug ist für den 06.–07.10. keine Hotelzahlung zu finden. Entweder über ein anderes Konto oder vorab bezahlt.
 Hotelrechnung beilegen und Betrag hier eintragen. Enthält sie Frühstück, den Anteil herausrechnen und oben in Block C das „F“ setzen.</t>
         </r>
       </text>
@@ -126,6 +126,19 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Hier den tatsächlich gezahlten Betrag eintragen.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I67" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Flug Rückreise, 89,98 €. Die Rechnung läuft auf die Coldewey Holding GmbH und die Zahlung steht nicht im privaten Kontoauszug — also hat die Firma direkt gezahlt.
+Hast du den Flug doch privat ausgelegt, diesen Abzug löschen.</t>
         </r>
       </text>
     </comment>
@@ -169,18 +182,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="135">
   <si>
     <t xml:space="preserve">Reisekostenabrechnung</t>
   </si>
   <si>
-    <t xml:space="preserve">London · 07.–08.10.2026 · Sätze siehe Blatt „Saetze 2026“</t>
+    <t xml:space="preserve">London · 06.–07.10.2026 · Sätze siehe Blatt „Saetze 2026“</t>
   </si>
   <si>
     <t xml:space="preserve">Firma</t>
   </si>
   <si>
-    <t xml:space="preserve">Coldewey Holding</t>
+    <t xml:space="preserve">Coldewey Holding GmbH, Im Zuckergarten 28, 55129 Mainz</t>
   </si>
   <si>
     <t xml:space="preserve">Gelb = ausfüllen</t>
@@ -189,7 +202,7 @@
     <t xml:space="preserve">Reisende/r</t>
   </si>
   <si>
-    <t xml:space="preserve">Sascha Coldewey</t>
+    <t xml:space="preserve">Sascha Elimar Coldewey</t>
   </si>
   <si>
     <t xml:space="preserve">Weiß = rechnet sich</t>
@@ -219,13 +232,13 @@
     <t xml:space="preserve">Reise von (Datum, Uhrzeit)</t>
   </si>
   <si>
-    <t xml:space="preserve">07.10.2026, __:__</t>
+    <t xml:space="preserve">06.10.2026, __:__</t>
   </si>
   <si>
     <t xml:space="preserve">Reise bis (Datum, Uhrzeit)</t>
   </si>
   <si>
-    <t xml:space="preserve">08.10.2026, __:__</t>
+    <t xml:space="preserve">07.10.2026, 22:05</t>
   </si>
   <si>
     <t xml:space="preserve">Abrechnung erstellt am</t>
@@ -249,201 +262,216 @@
     <t xml:space="preserve">Zelle I29</t>
   </si>
   <si>
+    <t xml:space="preserve">Flug Hinreise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frankfurt → London am 06.10., gezahlter Preis — die Rückreise ist mit 89,99 € bereits erfasst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelle I51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Übernachtung 07. auf 08.10., ohne Frühstücksanteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A · Fahrt mit eigenem Fahrzeug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strecke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fahrzeug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kilometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/km</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Im Zuckergarten 28 → FRA Terminal 3 und zurück</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pkw, je Kilometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe Fahrt eigenes Fahrzeug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B · Fahrtkosten und Transport mit Beleg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Art</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beschreibung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frankfurt → London, Beleg fehlt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flug Rückreise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LH 919 London LHR T2 → Frankfurt FRA T1, Rechnung 2026-B2B7-000199110 vom 24.08.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flughafen-Parken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parkhaus FRA Terminal 3, 06.–07.10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U-Bahn London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUL Ticket Machine, 7,00 GBP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TfL Nachzahlung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TFL Unpaid Fare, 26,00 GBP — siehe Hinweis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nahverkehr London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About Town Business Services, 3,15 GBP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About Town Business Services, 2,00 GBP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe Fahrtkosten mit Beleg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · Verpflegungsmehraufwand (Pauschale, kein Beleg nötig)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ort / Land</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abwesenheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pauschale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kürzung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An-/Abreisetag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe Verpflegungsmehraufwand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D · Übernachtung (mit Beleg, ohne Frühstücksanteil)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel / Ort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beleg-Nr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel London, Nacht 06. auf 07.10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beleg fehlt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe Übernachtung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E · Sonstige Reisenebenkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einreisegenehmigung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UKVI ETA, Pflicht für UK-Einreise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe sonstige Nebenkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ergebnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe A bis E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abzüglich Vorschuss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abzüglich direkt von der Firma bezahlt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zu erstatten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_______________________________</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ort, Datum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unterschrift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offene Punkte und bewusst nicht aufgenommene Positionen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OFFEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frankfurt → London am 06.10. fehlt. Die Opodo-Buchung 25549946153 deckt nur die Rückreise ab (LH 919, 89,99 €). Beleg der Hinreise nachreichen, Block B.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">89,98 € laut Rechnung 2026-B2B7-000199110. Rechnungsempfänger ist die Coldewey Holding GmbH mit ihrer USt-ID, und im privaten Kontoauszug ist keine Zahlung an Opodo oder eDreams — die Firma hat also direkt gezahlt. Der Betrag steht deshalb oben in Block B und wird unten wieder abgezogen: er gehört zu den Reisekosten, ist aber keine Auslage von dir. Stimmt das nicht, den Abzug löschen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fehlt im Kopf der Abrechnung. Ohne betrieblichen Anlass ist die Reise nicht absetzbar — Zweck und, wenn möglich, Gesprächspartner eintragen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nacht 06. auf 07.10., Betrag in Block D eintragen. Im Kontoauszug dieses Kontos ist die Zahlung nicht — Rechnung beilegen. Enthält sie Frühstück, den Anteil herausrechnen und in Block C das „F“ setzen, das kürzt die Pauschale um 13,20 €.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flug</t>
   </si>
   <si>
-    <t xml:space="preserve">Frankfurt → London → Frankfurt, gezahlter Preis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zelle I51</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Übernachtung 07. auf 08.10., ohne Frühstücksanteil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A · Fahrt mit eigenem Fahrzeug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Datum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strecke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fahrzeug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kilometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€/km</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07.10.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Im Zuckergarten 28 → FRA Terminal 3 und zurück</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pkw, je Kilometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summe Fahrt eigenes Fahrzeug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B · Fahrtkosten und Transport mit Beleg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Art</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beschreibung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frankfurt → London → Frankfurt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flughafen-Parken</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parkhaus FRA Terminal 3, 07.–08.10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">08.10.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U-Bahn London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUL Ticket Machine, 7,00 GBP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TfL Nachzahlung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TFL Unpaid Fare, 26,00 GBP — siehe Hinweis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nahverkehr London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">About Town Business Services, 3,15 GBP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">About Town Business Services, 2,00 GBP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summe Fahrtkosten mit Beleg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C · Verpflegungsmehraufwand (Pauschale, kein Beleg nötig)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ort / Land</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abwesenheit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pauschale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kürzung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An-/Abreisetag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summe Verpflegungsmehraufwand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D · Übernachtung (mit Beleg, ohne Frühstücksanteil)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel / Ort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beleg-Nr.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beleg fehlt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summe Übernachtung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E · Sonstige Reisenebenkosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06.10.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einreisegenehmigung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UKVI ETA, Pflicht für UK-Einreise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summe sonstige Nebenkosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ergebnis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summe A bis E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">abzüglich Vorschuss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">abzüglich direkt von der Firma bezahlt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zu erstatten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">_______________________________</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ort, Datum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unterschrift</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offene Punkte und bewusst nicht aufgenommene Positionen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OFFEN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reisedatum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Du hast 06. auf 07.10. genannt. Die Kartenumsätze sprechen für 07. auf 08.10.: Abflug Frankfurt „Pier J NonSchengen T3“ am 07.10., Rückflug „WH Smith Heathrow T2“ und Parkhaus-Ausfahrt am 08.10. Die Abrechnung steht auf 07.–08.10. — bitte prüfen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betrag in Block D eintragen. Im Kontoauszug dieses Kontos ist die Zahlung nicht — Rechnung beilegen. Enthält sie Frühstück, den Anteil herausrechnen und in Block C das „F“ setzen, das kürzt die Pauschale um 13,20 €.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Betrag in Block B eintragen. Hat die Firma direkt gezahlt, gehört er nicht hierher, sondern unten in „abzüglich direkt von der Firma bezahlt“.</t>
   </si>
   <si>
@@ -459,9 +487,6 @@
     <t xml:space="preserve">3 Buchungen über zusammen 9,81 € nicht eindeutig zuzuordnen. Prüfen.</t>
   </si>
   <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
     <t xml:space="preserve">UPS-Zoll 14 €</t>
   </si>
   <si>
@@ -472,6 +497,18 @@
   </si>
   <si>
     <t xml:space="preserve">Pret a Manger, Costa, Nazari Food, WH Smith: zusammen 43,74 €. Wird NICHT zusätzlich erstattet, die Verpflegungspauschale deckt das ab. Die Pauschale von 88 € liegt deutlich darüber.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belegdaten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Daten in den Blöcken B und E sind die Kauftage. Im Kontoauszug stehen sie ein bis zwei Tage später, weil der Händler den Kartenumsatz erst dann einreicht. Deshalb sah der Auszug zunächst nach 07.–08.10. aus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorsteuer Flug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grenzüberschreitende Flüge sind in Deutschland nicht umsatzsteuerpflichtig. Aus den 89,99 € ist keine Vorsteuer zu ziehen, der Betrag wird brutto gebucht.</t>
   </si>
   <si>
     <t xml:space="preserve">Pauschalen 2026</t>
@@ -1172,7 +1209,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1547,13 +1584,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D30" s="19"/>
       <c r="E30" s="19"/>
@@ -1561,12 +1598,12 @@
       <c r="G30" s="19"/>
       <c r="H30" s="19"/>
       <c r="I30" s="21" t="n">
-        <v>86</v>
+        <v>89.98</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>48</v>
@@ -1580,14 +1617,14 @@
       <c r="G31" s="19"/>
       <c r="H31" s="19"/>
       <c r="I31" s="21" t="n">
-        <v>8.26</v>
+        <v>86</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B32" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>50</v>
       </c>
       <c r="C32" s="4" t="s">
@@ -1599,14 +1636,14 @@
       <c r="G32" s="19"/>
       <c r="H32" s="19"/>
       <c r="I32" s="21" t="n">
-        <v>30.68</v>
+        <v>8.26</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="22" t="s">
         <v>52</v>
       </c>
       <c r="C33" s="4" t="s">
@@ -1618,18 +1655,18 @@
       <c r="G33" s="19"/>
       <c r="H33" s="19"/>
       <c r="I33" s="21" t="n">
-        <v>3.73</v>
+        <v>30.68</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D34" s="19"/>
       <c r="E34" s="19"/>
@@ -1637,18 +1674,18 @@
       <c r="G34" s="19"/>
       <c r="H34" s="19"/>
       <c r="I34" s="21" t="n">
-        <v>3.72</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D35" s="19"/>
       <c r="E35" s="19"/>
@@ -1656,24 +1693,32 @@
       <c r="G35" s="19"/>
       <c r="H35" s="19"/>
       <c r="I35" s="21" t="n">
-        <v>2.36</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
+      <c r="A36" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>56</v>
+      </c>
       <c r="D36" s="19"/>
       <c r="E36" s="19"/>
       <c r="F36" s="19"/>
       <c r="G36" s="19"/>
       <c r="H36" s="19"/>
-      <c r="I36" s="21"/>
+      <c r="I36" s="21" t="n">
+        <v>2.36</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="17" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
@@ -1683,12 +1728,12 @@
       <c r="H37" s="16"/>
       <c r="I37" s="18" t="n">
         <f aca="false">SUM(I29:I36)</f>
-        <v>134.75</v>
+        <v>224.73</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -1704,25 +1749,25 @@
         <v>32</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I40" s="7" t="s">
         <v>24</v>
@@ -1733,10 +1778,10 @@
         <v>37</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D41" s="15" t="n">
         <f aca="false">IF($A41="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B41,'Saetze 2026'!$B$5:$B$7,0),MATCH($C41,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
@@ -1756,13 +1801,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D42" s="15" t="n">
         <f aca="false">IF($A42="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B42,'Saetze 2026'!$B$5:$B$7,0),MATCH($C42,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
@@ -1863,7 +1908,7 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="16"/>
       <c r="B47" s="17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
@@ -1878,7 +1923,7 @@
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -1894,10 +1939,10 @@
         <v>32</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I50" s="7" t="s">
         <v>24</v>
@@ -1908,10 +1953,10 @@
         <v>37</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D51" s="19"/>
       <c r="E51" s="19"/>
@@ -1945,7 +1990,7 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="16"/>
       <c r="B54" s="17" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C54" s="16"/>
       <c r="D54" s="16"/>
@@ -1960,7 +2005,7 @@
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -1987,13 +2032,13 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D58" s="19"/>
       <c r="E58" s="19"/>
@@ -2040,7 +2085,7 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="16"/>
       <c r="B62" s="17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C62" s="16"/>
       <c r="D62" s="16"/>
@@ -2055,7 +2100,7 @@
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -2068,29 +2113,31 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I65" s="24" t="n">
         <f aca="false">I25+I37+I47+I54+I62</f>
-        <v>267.98</v>
+        <v>357.96</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="25" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I66" s="21"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="I67" s="21"/>
+        <v>82</v>
+      </c>
+      <c r="I67" s="21" t="n">
+        <v>89.98</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="26"/>
       <c r="B68" s="27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C68" s="26"/>
       <c r="D68" s="26"/>
@@ -2105,23 +2152,23 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E71" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -2134,13 +2181,13 @@
     </row>
     <row r="76" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="29" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B76" s="30" t="s">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="C76" s="31" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D76" s="31"/>
       <c r="E76" s="31"/>
@@ -2150,31 +2197,31 @@
       <c r="I76" s="31"/>
     </row>
     <row r="77" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="B77" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="C77" s="31" t="s">
+      <c r="A77" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="D77" s="31"/>
-      <c r="E77" s="31"/>
-      <c r="F77" s="31"/>
-      <c r="G77" s="31"/>
-      <c r="H77" s="31"/>
-      <c r="I77" s="31"/>
+      <c r="B77" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C77" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D77" s="34"/>
+      <c r="E77" s="34"/>
+      <c r="F77" s="34"/>
+      <c r="G77" s="34"/>
+      <c r="H77" s="34"/>
+      <c r="I77" s="34"/>
     </row>
     <row r="78" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="29" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B78" s="30" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="C78" s="31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D78" s="31"/>
       <c r="E78" s="31"/>
@@ -2183,15 +2230,15 @@
       <c r="H78" s="31"/>
       <c r="I78" s="31"/>
     </row>
-    <row r="79" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="29" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B79" s="30" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C79" s="31" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D79" s="31"/>
       <c r="E79" s="31"/>
@@ -2200,15 +2247,15 @@
       <c r="H79" s="31"/>
       <c r="I79" s="31"/>
     </row>
-    <row r="80" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="29" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B80" s="30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C80" s="31" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D80" s="31"/>
       <c r="E80" s="31"/>
@@ -2217,42 +2264,110 @@
       <c r="H80" s="31"/>
       <c r="I80" s="31"/>
     </row>
-    <row r="81" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B81" s="33" t="s">
+    <row r="81" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B81" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="C81" s="34" t="s">
+      <c r="C81" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="D81" s="34"/>
-      <c r="E81" s="34"/>
-      <c r="F81" s="34"/>
-      <c r="G81" s="34"/>
-      <c r="H81" s="34"/>
-      <c r="I81" s="34"/>
-    </row>
-    <row r="82" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B82" s="33" t="s">
+      <c r="D81" s="31"/>
+      <c r="E81" s="31"/>
+      <c r="F81" s="31"/>
+      <c r="G81" s="31"/>
+      <c r="H81" s="31"/>
+      <c r="I81" s="31"/>
+    </row>
+    <row r="82" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B82" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="C82" s="34" t="s">
+      <c r="C82" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="D82" s="34"/>
-      <c r="E82" s="34"/>
-      <c r="F82" s="34"/>
-      <c r="G82" s="34"/>
-      <c r="H82" s="34"/>
-      <c r="I82" s="34"/>
+      <c r="D82" s="31"/>
+      <c r="E82" s="31"/>
+      <c r="F82" s="31"/>
+      <c r="G82" s="31"/>
+      <c r="H82" s="31"/>
+      <c r="I82" s="31"/>
+    </row>
+    <row r="83" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B83" s="33" t="s">
+        <v>101</v>
+      </c>
+      <c r="C83" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="D83" s="34"/>
+      <c r="E83" s="34"/>
+      <c r="F83" s="34"/>
+      <c r="G83" s="34"/>
+      <c r="H83" s="34"/>
+      <c r="I83" s="34"/>
+    </row>
+    <row r="84" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B84" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="C84" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="D84" s="34"/>
+      <c r="E84" s="34"/>
+      <c r="F84" s="34"/>
+      <c r="G84" s="34"/>
+      <c r="H84" s="34"/>
+      <c r="I84" s="34"/>
+    </row>
+    <row r="85" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B85" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="C85" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="D85" s="34"/>
+      <c r="E85" s="34"/>
+      <c r="F85" s="34"/>
+      <c r="G85" s="34"/>
+      <c r="H85" s="34"/>
+      <c r="I85" s="34"/>
+    </row>
+    <row r="86" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B86" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="C86" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="D86" s="34"/>
+      <c r="E86" s="34"/>
+      <c r="F86" s="34"/>
+      <c r="G86" s="34"/>
+      <c r="H86" s="34"/>
+      <c r="I86" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="52">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="B4:E4"/>
@@ -2301,6 +2416,10 @@
     <mergeCell ref="C80:I80"/>
     <mergeCell ref="C81:I81"/>
     <mergeCell ref="C82:I82"/>
+    <mergeCell ref="C83:I83"/>
+    <mergeCell ref="C84:I84"/>
+    <mergeCell ref="C85:I85"/>
+    <mergeCell ref="C86:I86"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C21:C24" type="list">
@@ -2348,43 +2467,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="25" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C5" s="36" t="n">
         <v>28</v>
@@ -2399,15 +2518,15 @@
         <v>0</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C6" s="36" t="n">
         <v>66</v>
@@ -2427,10 +2546,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>52</v>
@@ -2450,12 +2569,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B10" s="37" t="n">
         <v>0.2</v>
@@ -2463,7 +2582,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="25" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="B11" s="37" t="n">
         <v>0.4</v>
@@ -2471,7 +2590,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B12" s="37" t="n">
         <v>0.4</v>
@@ -2479,7 +2598,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2492,7 +2611,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="C16" s="38" t="n">
         <v>0.2</v>
@@ -2500,7 +2619,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="25" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="C17" s="38" t="n">
         <v>0.05</v>
@@ -2508,42 +2627,42 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reisekosten London: UPS-Hinweis korrigiert
Der UPS-Beleg nennt 11,23 EUR, nicht 14 EUR, und die Zustellung war am
26.08.2026 - sechs Wochen vor der Reise. Hinweis in der Abrechnung
entsprechend praezisiert.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-21-reisekosten-london-coldewey-holding.xlsx
+++ b/10_Output/2026-10-21-reisekosten-london-coldewey-holding.xlsx
@@ -487,10 +487,10 @@
     <t xml:space="preserve">3 Buchungen über zusammen 9,81 € nicht eindeutig zuzuordnen. Prüfen.</t>
   </si>
   <si>
-    <t xml:space="preserve">UPS-Zoll 14 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gehört nicht in die Reisekostenabrechnung. Einfuhrabgaben für ein Paket sind eine eigene Betriebsausgabe und werden separat gebucht. Im Kontoauszug nicht enthalten, also wohl bar bezahlt — Beleg aufheben.</t>
+    <t xml:space="preserve">UPS-Einfuhrabgaben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11,23 €, Paket zugestellt am 26.08.2026 — sechs Wochen vor dieser Reise und ohne Bezug zu ihr. Gehört nicht in die Reisekostenabrechnung, sondern als eigene Betriebsausgabe gebucht, falls die Sendung betrieblich war. Im privaten Kontoauszug ist die Zahlung nicht zu finden.</t>
   </si>
   <si>
     <t xml:space="preserve">Essen in London</t>

</xml_diff>